<commit_message>
[REVIEW] Рецензування BUG-001…007, README, task-board
</commit_message>
<xml_diff>
--- a/docs/sprint3/execution-log.xlsx
+++ b/docs/sprint3/execution-log.xlsx
@@ -4451,7 +4451,7 @@
       <c r="J56" s="16" t="n"/>
       <c r="K56" s="16" t="inlineStr">
         <is>
-          <t>Chrome ВЕРСІЯ_CHROME</t>
+          <t>Chrome</t>
         </is>
       </c>
       <c r="L56" s="16" t="inlineStr">
@@ -4522,7 +4522,7 @@
       <c r="J57" s="16" t="n"/>
       <c r="K57" s="16" t="inlineStr">
         <is>
-          <t>Firefox ВЕРСІЯ_FIREFOX</t>
+          <t>Firefox</t>
         </is>
       </c>
       <c r="L57" s="16" t="inlineStr">
@@ -4593,7 +4593,7 @@
       <c r="J58" s="16" t="n"/>
       <c r="K58" s="16" t="inlineStr">
         <is>
-          <t>Chrome ВЕРСІЯ_CHROME</t>
+          <t>Chrome</t>
         </is>
       </c>
       <c r="L58" s="16" t="inlineStr">
@@ -4664,7 +4664,7 @@
       <c r="J59" s="16" t="n"/>
       <c r="K59" s="16" t="inlineStr">
         <is>
-          <t>Firefox ВЕРСІЯ_FIREFOX</t>
+          <t>Firefox</t>
         </is>
       </c>
       <c r="L59" s="16" t="inlineStr">
@@ -4965,7 +4965,7 @@
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Chrome ВЕРСІЯ_CHROME</t>
+          <t>Google Chrome, поточна стабільна версія станом на 25–28.10.2026</t>
         </is>
       </c>
     </row>
@@ -4977,7 +4977,7 @@
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>Firefox ВЕРСІЯ_FIREFOX</t>
+          <t>Mozilla Firefox, поточна стабільна версія станом на 28.10.2026 (TC-052, TC-053)</t>
         </is>
       </c>
     </row>
@@ -4989,7 +4989,7 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Windows ВЕРСІЯ_WINDOWS</t>
+          <t>Windows 11</t>
         </is>
       </c>
     </row>
@@ -5080,12 +5080,12 @@
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Коміт restful-booker-platform</t>
+          <t>Версія restful-booker-platform</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>КОМІТ</t>
+          <t>ZIP-архів гілки trunk (без git-коміту), завантажено перед Run 1</t>
         </is>
       </c>
     </row>

</xml_diff>